<commit_message>
Add recent emails feature
</commit_message>
<xml_diff>
--- a/companies.xlsx
+++ b/companies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Geelcom Toshiba\Downloads\Sir AI Telegram Bot V1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867EE4BF-54C7-4D9E-B510-62C48D90DD73}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789A0385-B9AA-47CD-B300-4CD19C748B64}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{E8DFB9B0-C094-44BF-B090-3C96ECD70C43}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12111" uniqueCount="6092">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12112" uniqueCount="6093">
   <si>
     <t>Email</t>
   </si>
@@ -18323,6 +18323,9 @@
   </si>
   <si>
     <t>مراقب جودة وسلامة - أخصائية موارد بشرية، محاسبة، مساعد إداري - مدير مخاطر</t>
+  </si>
+  <si>
+    <t>تاريخ الإضافة</t>
   </si>
 </sst>
 </file>
@@ -18453,12 +18456,14 @@
     <cellStyle name="ارتباط تشعبي" xfId="1" builtinId="8"/>
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="8">
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -18503,146 +18508,32 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -18956,15 +18847,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39160EC8-75D0-45BF-8D14-DAE9F6D10B5D}">
-  <dimension ref="A1:D3089"/>
+  <dimension ref="A1:E3089"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="35.3984375" customWidth="1"/>
     <col min="3" max="3" width="31.09765625" customWidth="1"/>
     <col min="4" max="4" width="31.69921875" customWidth="1"/>
+    <col min="5" max="5" width="18.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.4" thickBot="1">
+    <row r="1" spans="1:5" ht="14.4" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -18977,8 +18869,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="180" thickBot="1">
+      <c r="E1" s="1" t="s">
+        <v>6092</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="180" thickBot="1">
       <c r="A2" s="2" t="s">
         <v>1910</v>
       </c>
@@ -18992,7 +18887,7 @@
         <v>6020</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="262.8" thickBot="1">
+    <row r="3" spans="1:5" ht="262.8" thickBot="1">
       <c r="A3" s="2" t="s">
         <v>3135</v>
       </c>
@@ -19006,7 +18901,7 @@
         <v>6022</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="409.6" thickBot="1">
+    <row r="4" spans="1:5" ht="409.6" thickBot="1">
       <c r="A4" s="2" t="s">
         <v>2059</v>
       </c>
@@ -19020,7 +18915,7 @@
         <v>6024</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="83.4" thickBot="1">
+    <row r="5" spans="1:5" ht="83.4" thickBot="1">
       <c r="A5" s="2" t="s">
         <v>2812</v>
       </c>
@@ -19034,7 +18929,7 @@
         <v>6026</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="97.2" thickBot="1">
+    <row r="6" spans="1:5" ht="97.2" thickBot="1">
       <c r="A6" s="2" t="s">
         <v>2406</v>
       </c>
@@ -19048,7 +18943,7 @@
         <v>6025</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="14.4" thickBot="1">
+    <row r="7" spans="1:5" ht="14.4" thickBot="1">
       <c r="A7" s="2" t="s">
         <v>4259</v>
       </c>
@@ -19062,7 +18957,7 @@
         <v>6028</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="14.4" thickBot="1">
+    <row r="8" spans="1:5" ht="14.4" thickBot="1">
       <c r="A8" s="2" t="s">
         <v>2657</v>
       </c>
@@ -19076,7 +18971,7 @@
         <v>6029</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="69.599999999999994" thickBot="1">
+    <row r="9" spans="1:5" ht="69.599999999999994" thickBot="1">
       <c r="A9" s="2" t="s">
         <v>1994</v>
       </c>
@@ -19090,7 +18985,7 @@
         <v>6030</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="42" thickBot="1">
+    <row r="10" spans="1:5" ht="42" thickBot="1">
       <c r="A10" s="2" t="s">
         <v>2885</v>
       </c>
@@ -19104,7 +18999,7 @@
         <v>6031</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28.2" thickBot="1">
+    <row r="11" spans="1:5" ht="28.2" thickBot="1">
       <c r="A11" s="2" t="s">
         <v>915</v>
       </c>
@@ -19118,7 +19013,7 @@
         <v>6032</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="97.2" thickBot="1">
+    <row r="12" spans="1:5" ht="97.2" thickBot="1">
       <c r="A12" s="2" t="s">
         <v>1840</v>
       </c>
@@ -19132,7 +19027,7 @@
         <v>6035</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="28.2" thickBot="1">
+    <row r="13" spans="1:5" ht="28.2" thickBot="1">
       <c r="A13" s="2" t="s">
         <v>1998</v>
       </c>
@@ -19146,7 +19041,7 @@
         <v>6036</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="42" thickBot="1">
+    <row r="14" spans="1:5" ht="42" thickBot="1">
       <c r="A14" s="2" t="s">
         <v>3169</v>
       </c>
@@ -19160,7 +19055,7 @@
         <v>6037</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="14.4" thickBot="1">
+    <row r="15" spans="1:5" ht="14.4" thickBot="1">
       <c r="A15" s="2" t="s">
         <v>1515</v>
       </c>
@@ -19174,7 +19069,7 @@
         <v>6038</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="83.4" thickBot="1">
+    <row r="16" spans="1:5" ht="83.4" thickBot="1">
       <c r="A16" s="2" t="s">
         <v>324</v>
       </c>
@@ -61491,7 +61386,7 @@
       <c r="D3068" s="6"/>
     </row>
     <row r="3069" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A3069" s="2" t="s">
+      <c r="A3069" s="4" t="s">
         <v>211</v>
       </c>
       <c r="B3069" s="2" t="s">
@@ -61743,14 +61638,6 @@
   </sheetData>
   <autoFilter ref="A1:A3167" xr:uid="{0A1E0DAA-A8ED-49EF-A4F6-6D96590D266E}"/>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A3090:A1048576 A1:A701">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
-  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A1283" r:id="rId1" xr:uid="{D537246E-8512-472A-B8CA-0A3388A8AC59}"/>
     <hyperlink ref="A745" r:id="rId2" xr:uid="{7AE35F11-BFE0-4E04-BB7D-F2365B0C5A0F}"/>
@@ -61771,8 +61658,9 @@
     <hyperlink ref="A3067" r:id="rId17" display="https://www.google.com/search?q=https%3A%2F%2Fwww.sbm.com&amp;authuser=4" xr:uid="{63F952C0-F4F1-4F24-89D5-FCFDFDCE0A68}"/>
     <hyperlink ref="A2318" r:id="rId18" xr:uid="{00718BA7-AFB1-456B-A4CD-E8086F69E725}"/>
     <hyperlink ref="A3068" r:id="rId19" display="https://www.google.com/search?q=https%3A%2F%2Fwww.subsea7.com&amp;authuser=4" xr:uid="{62ADC037-F07E-468B-943C-07BBD320E9E1}"/>
+    <hyperlink ref="A3069" r:id="rId20" xr:uid="{BD554AE0-9154-4B96-ACF9-77EF4581077A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new email notifications
</commit_message>
<xml_diff>
--- a/companies.xlsx
+++ b/companies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Geelcom Toshiba\Downloads\Sir AI Telegram Bot V1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAD54E7-1E5C-492C-B2F0-9DF02D446939}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C36E86E-AB33-4EFF-9EEF-F806F61D646A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{E8DFB9B0-C094-44BF-B090-3C96ECD70C43}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12116" uniqueCount="6094">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12112" uniqueCount="6093">
   <si>
     <t>Email</t>
   </si>
@@ -18326,9 +18326,6 @@
   </si>
   <si>
     <t>تاريخ الإضافة</t>
-  </si>
-  <si>
-    <t>tha@</t>
   </si>
 </sst>
 </file>
@@ -18406,7 +18403,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -18429,23 +18426,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFC4C7C5"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFC4C7C5"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -18466,12 +18452,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ارتباط تشعبي" xfId="1" builtinId="8"/>
@@ -18787,7 +18767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39160EC8-75D0-45BF-8D14-DAE9F6D10B5D}">
-  <dimension ref="A1:E3090"/>
+  <dimension ref="A1:E3089"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="35.3984375" customWidth="1"/>
@@ -61574,22 +61554,8 @@
         <v>6011</v>
       </c>
       <c r="D3089" s="6"/>
-    </row>
-    <row r="3090" spans="1:5">
-      <c r="A3090" s="9" t="s">
-        <v>6093</v>
-      </c>
-      <c r="B3090" s="8" t="s">
-        <v>884</v>
-      </c>
-      <c r="C3090" s="8" t="s">
-        <v>884</v>
-      </c>
-      <c r="D3090" t="s">
-        <v>884</v>
-      </c>
-      <c r="E3090" s="7">
-        <v>46243</v>
+      <c r="E3089" s="7">
+        <v>46242</v>
       </c>
     </row>
   </sheetData>
@@ -61616,9 +61582,8 @@
     <hyperlink ref="A2318" r:id="rId18" xr:uid="{00718BA7-AFB1-456B-A4CD-E8086F69E725}"/>
     <hyperlink ref="A3068" r:id="rId19" display="https://www.google.com/search?q=https%3A%2F%2Fwww.subsea7.com&amp;authuser=4" xr:uid="{62ADC037-F07E-468B-943C-07BBD320E9E1}"/>
     <hyperlink ref="A3069" r:id="rId20" xr:uid="{BD554AE0-9154-4B96-ACF9-77EF4581077A}"/>
-    <hyperlink ref="A3090" r:id="rId21" xr:uid="{2FEE1288-F86B-47FF-B5CC-E0E6E1BBE688}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId22"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>